<commit_message>
Update agile tracking file
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Agile_File_v0.1.xlsx
+++ b/Agile_File_v0.1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7A1D06736B73C21B/Documents/GTA Vice City User Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harsh\OneDrive\Documents\GTA Vice City User Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{91776049-14DB-4AE1-9468-085EB89BA1FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7204949C-49D8-4AB4-A2DA-15A5D973D3FC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2C705A2-F2DE-4723-9BF6-1516E9D3D759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="93">
   <si>
     <t>Planned Sprint</t>
   </si>
@@ -311,6 +311,9 @@
   </si>
   <si>
     <t>completed</t>
+  </si>
+  <si>
+    <t>Harsh Joshi</t>
   </si>
 </sst>
 </file>
@@ -816,10 +819,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -1170,7 +1169,9 @@
       <c r="F2" s="52" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="2"/>
+      <c r="G2" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H2" s="5" t="s">
         <v>91</v>
       </c>
@@ -1192,7 +1193,9 @@
       <c r="F3" s="54" t="s">
         <v>69</v>
       </c>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H3" s="5" t="s">
         <v>91</v>
       </c>
@@ -1214,7 +1217,9 @@
       <c r="F4" s="52" t="s">
         <v>71</v>
       </c>
-      <c r="G4" s="2"/>
+      <c r="G4" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H4" s="5" t="s">
         <v>91</v>
       </c>
@@ -1236,7 +1241,9 @@
       <c r="F5" s="52" t="s">
         <v>73</v>
       </c>
-      <c r="G5" s="2"/>
+      <c r="G5" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H5" s="2" t="s">
         <v>91</v>
       </c>
@@ -1258,7 +1265,9 @@
       <c r="F6" s="52" t="s">
         <v>75</v>
       </c>
-      <c r="G6" s="2"/>
+      <c r="G6" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H6" s="5" t="s">
         <v>91</v>
       </c>
@@ -1280,7 +1289,9 @@
       <c r="F7" s="52" t="s">
         <v>77</v>
       </c>
-      <c r="G7" s="2"/>
+      <c r="G7" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H7" s="5" t="s">
         <v>91</v>
       </c>
@@ -1302,7 +1313,9 @@
       <c r="F8" s="52" t="s">
         <v>79</v>
       </c>
-      <c r="G8" s="2"/>
+      <c r="G8" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H8" s="5" t="s">
         <v>91</v>
       </c>
@@ -1324,7 +1337,9 @@
       <c r="F9" s="52" t="s">
         <v>49</v>
       </c>
-      <c r="G9" s="2"/>
+      <c r="G9" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H9" s="5" t="s">
         <v>91</v>
       </c>
@@ -1346,7 +1361,9 @@
       <c r="F10" s="52" t="s">
         <v>80</v>
       </c>
-      <c r="G10" s="2"/>
+      <c r="G10" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H10" s="5" t="s">
         <v>91</v>
       </c>
@@ -1368,7 +1385,9 @@
       <c r="F11" s="52" t="s">
         <v>82</v>
       </c>
-      <c r="G11" s="2"/>
+      <c r="G11" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H11" s="2" t="s">
         <v>91</v>
       </c>
@@ -1390,7 +1409,9 @@
       <c r="F12" s="52" t="s">
         <v>84</v>
       </c>
-      <c r="G12" s="2"/>
+      <c r="G12" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H12" s="2" t="s">
         <v>91</v>
       </c>
@@ -1412,7 +1433,9 @@
       <c r="F13" s="52" t="s">
         <v>67</v>
       </c>
-      <c r="G13" s="2"/>
+      <c r="G13" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H13" s="2" t="s">
         <v>91</v>
       </c>
@@ -1434,7 +1457,9 @@
       <c r="F14" s="52" t="s">
         <v>86</v>
       </c>
-      <c r="G14" s="2"/>
+      <c r="G14" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H14" s="2" t="s">
         <v>91</v>
       </c>
@@ -1456,7 +1481,9 @@
       <c r="F15" s="52" t="s">
         <v>50</v>
       </c>
-      <c r="G15" s="2"/>
+      <c r="G15" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H15" s="2" t="s">
         <v>91</v>
       </c>
@@ -1478,7 +1505,9 @@
       <c r="F16" s="52" t="s">
         <v>89</v>
       </c>
-      <c r="G16" s="2"/>
+      <c r="G16" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H16" s="2" t="s">
         <v>91</v>
       </c>
@@ -1500,7 +1529,9 @@
       <c r="F17" s="52" t="s">
         <v>54</v>
       </c>
-      <c r="G17" s="2"/>
+      <c r="G17" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="H17" s="2" t="s">
         <v>91</v>
       </c>

</xml_diff>